<commit_message>
PMAS reports: add cycle result samples and update test parameter workbook
</commit_message>
<xml_diff>
--- a/Codex_PMAS_WPF/Reports/테스트 파라메터.xlsx
+++ b/Codex_PMAS_WPF/Reports/테스트 파라메터.xlsx
@@ -9,17 +9,18 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="29010" windowHeight="13095"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25605" windowHeight="11970"/>
   </bookViews>
   <sheets>
     <sheet name="CycleTest Params" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
   <si>
     <t>테스트 파라메터</t>
   </si>
@@ -48,13 +49,7 @@
     <t>Move Distance (mm)</t>
   </si>
   <si>
-    <t>8388608</t>
-  </si>
-  <si>
     <t>Velocity (mm/s)</t>
-  </si>
-  <si>
-    <t>48933546</t>
   </si>
   <si>
     <t>Acceleration (mm/s^2)</t>
@@ -139,11 +134,13 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>0.1 s</t>
+    <t>0.05 도</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>0.05 도</t>
+    <t>0.1 s
+Elmo와 Sigmatek 
+Jerk 수치는 *1000 차이남</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -221,19 +218,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -537,22 +545,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="26" style="6" customWidth="1"/>
+    <col min="3" max="3" width="20" style="2" customWidth="1"/>
+    <col min="4" max="4" width="26" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -560,197 +570,228 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="1"/>
+      <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+    </row>
+    <row r="6" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="6">
+        <v>8388608</v>
+      </c>
+      <c r="C6" s="6">
+        <v>360</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="B7" s="6">
+        <v>48933546</v>
+      </c>
+      <c r="C7" s="7">
+        <v>2100</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="6">
+        <v>4893354600</v>
+      </c>
+      <c r="C8" s="7">
+        <v>210000</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="7">
+        <v>210000</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="3" t="s">
+    <row r="10" spans="1:4" s="9" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="B10" s="6">
+        <v>48933546000</v>
+      </c>
+      <c r="C10" s="7">
+        <v>2100</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+    </row>
+    <row r="12" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="6">
+        <v>1165</v>
+      </c>
+      <c r="C12" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="3">
-        <v>48933546000</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="3" t="s">
+    <row r="13" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+    </row>
+    <row r="14" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="3"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="3">
-        <v>1165</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="3" t="s">
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+    </row>
+    <row r="15" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="3"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="B15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+    </row>
+    <row r="16" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B16" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="3"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+    </row>
+    <row r="17" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="3"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="B17" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="3"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="C17" s="6"/>
+      <c r="D17" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="3" t="s">
+    </row>
+    <row r="18" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="B18" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="C18" s="6"/>
+      <c r="D18" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="3" t="s">
+    </row>
+    <row r="19" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="B19" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="B20" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>30</v>
+      <c r="B21" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(pmas): add cycle result workbooks and update test parameter sheet
</commit_message>
<xml_diff>
--- a/Codex_PMAS_WPF/Reports/테스트 파라메터.xlsx
+++ b/Codex_PMAS_WPF/Reports/테스트 파라메터.xlsx
@@ -15,12 +15,11 @@
     <sheet name="CycleTest Params" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="39">
   <si>
     <t>테스트 파라메터</t>
   </si>
@@ -34,9 +33,6 @@
     <t>항목</t>
   </si>
   <si>
-    <t>값</t>
-  </si>
-  <si>
     <t>비고</t>
   </si>
   <si>
@@ -116,10 +112,6 @@
   </si>
   <si>
     <t>Request 1ms system timer resolution</t>
-  </si>
-  <si>
-    <t>350 RPM</t>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>23 bit</t>
@@ -138,9 +130,21 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
+    <t>P-MAS</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>SIGMATEK</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>350 RPM / 2100 RPS</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
     <t>0.1 s
-Elmo와 Sigmatek 
-Jerk 수치는 *1000 차이남</t>
+Sigmatek 
+Jerk 수치는 /1000 된 수치</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -226,8 +230,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -243,6 +245,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -555,12 +559,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -570,220 +574,242 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1" t="s">
+    </row>
+    <row r="5" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="4">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-    </row>
-    <row r="6" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="B6" s="4">
+        <v>8388608</v>
+      </c>
+      <c r="C6" s="4">
+        <v>360</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="6">
-        <v>8388608</v>
-      </c>
-      <c r="C6" s="6">
-        <v>360</v>
-      </c>
-      <c r="D6" s="6" t="s">
+      <c r="B7" s="4">
+        <v>48933546</v>
+      </c>
+      <c r="C7" s="5">
+        <v>2100</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="4">
+        <v>4893354600</v>
+      </c>
+      <c r="C8" s="5">
+        <v>210000</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="5">
+        <v>210000</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="6">
-        <v>48933546</v>
-      </c>
-      <c r="C7" s="7">
+    <row r="10" spans="1:4" s="7" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4">
+        <v>48933546000</v>
+      </c>
+      <c r="C10" s="5">
         <v>2100</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="6">
-        <v>4893354600</v>
-      </c>
-      <c r="C8" s="7">
-        <v>210000</v>
-      </c>
-      <c r="D8" s="6" t="s">
+      <c r="D10" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="4">
+        <v>1165</v>
+      </c>
+      <c r="C12" s="5">
+        <v>0.05</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="7">
-        <v>210000</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" s="9" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="6">
-        <v>48933546000</v>
-      </c>
-      <c r="C10" s="7">
-        <v>2100</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-    </row>
-    <row r="12" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+    <row r="13" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="6">
-        <v>1165</v>
-      </c>
-      <c r="C12" s="7">
-        <v>0.05</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="C14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" s="4"/>
+    </row>
+    <row r="16" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-    </row>
-    <row r="14" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="C16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="17" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="C17" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6" t="s">
+    </row>
+    <row r="18" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6" t="s">
+    </row>
+    <row r="19" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="B19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+    </row>
+    <row r="21" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>